<commit_message>
Reporte automatico abril 2026 generado por n8n
</commit_message>
<xml_diff>
--- a/reportes/Reporte_abril_2026.xlsx
+++ b/reportes/Reporte_abril_2026.xlsx
@@ -11898,7 +11898,7 @@
     <row r="50" ht="52" customHeight="1">
       <c r="B50" s="73" t="inlineStr">
         <is>
-          <t>Seducete redujo gasto en 7.6% (de $5.5M a $5.1M) pero también bajó resultados en 14.1% (de 35,423 a 30,410), indicando ineficiencia en la optimización. La campaña de conversión web absorbe 86.6% del presupuesto con ROAS crítico de 0.46 promedio, requiriendo restructuración inmediata.</t>
+          <t>Seducete redujo gasto en 7.6% (CLP 419.421) en abril pero también bajó resultados 14.1% (5.013 menos conversiones). La caída más crítica está en campañas de conversión web, donde el ROAS promedio es 0.27, indicando pérdida de eficiencia en el funnel.</t>
         </is>
       </c>
     </row>
@@ -11912,34 +11912,34 @@
     <row r="53" ht="50" customHeight="1">
       <c r="B53" s="74" t="inlineStr">
         <is>
-          <t>✦ OPORTUNIDAD  Anuncio de Cursos Presenciales supera en eficiencia</t>
+          <t>✦ OPORTUNIDAD  Anuncio Cursos Presenciales con mejor CPC</t>
         </is>
       </c>
       <c r="F53" s="75" t="inlineStr">
         <is>
-          <t>El anuncio 'Tráfico Cursos Presenciales 03-07' logró costo de $47 por resultado vs $59 del otro anuncio, representando 20% menos inversión. Con CTR de 1.7% mantiene buena tracción incluso con volumen similar de 1,890 resultados.</t>
+          <t>El anuncio 'Tráfico Cursos Presenciales 03-07' generó 1.890 resultados con CPC de CLP 47, 20% más eficiente que 'Tráfico Instagram Academia' (CLP 59). Sin embargo, bajó 2.3% en resultados respecto a marzo (1.847 vs 1.890).</t>
         </is>
       </c>
       <c r="M53" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Aumentar presupuesto del anuncio de Cursos Presenciales en 30% esta semana, reduciendo proporcionalmente el anuncio de Academia Gratuita.</t>
+          <t>→ Acción: Aumentar presupuesto del anuncio de Cursos Presenciales a CLP 120.000 y reducir el de Academia a CLP 75.000 para marzo de eficiencia.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="50" customHeight="1">
       <c r="B54" s="77" t="inlineStr">
         <is>
-          <t>⚠ ALERTA  Caída en resultados del anuncio principal</t>
+          <t>⚠ ALERTA  Caída en resultados de Academia Instagram</t>
         </is>
       </c>
       <c r="F54" s="75" t="inlineStr">
         <is>
-          <t>El anuncio 'Tráfico Instagram Academia Cursos Gratuitos' bajó de 1,546 a 1,775 resultados (15% aumento) pero con costo subido a $59, generando ineficiencia. El hold50 bajo de 5.8% sugiere contenido poco retentivo.</t>
+          <t>El anuncio 'Tráfico Instagram Academia Cursos Gratuitos' cayó 14.8% (1.775 vs 1.546 en marzo) con aumento de CPC de CLP 59. El hold50 de 5.8% sugiere abandono en video.</t>
         </is>
       </c>
       <c r="M54" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Testear 2 variantes de copy con hooks más fuertes enfocados en beneficio inmediato de cursos gratuitos esta semana.</t>
+          <t>→ Acción: Probar creativo de video más corto (primeros 3 segundos) y agregar subtítulos con oferta clara para mejorar hold50.</t>
         </is>
       </c>
     </row>
@@ -11953,34 +11953,34 @@
     <row r="57" ht="50" customHeight="1">
       <c r="B57" s="77" t="inlineStr">
         <is>
-          <t>⚠ ALERTA  Anuncio Esmaltado Permanente con ROAS catastrófico</t>
+          <t>⚠ ALERTA  Esmaltado Permanente con CPC descontrolado</t>
         </is>
       </c>
       <c r="F57" s="75" t="inlineStr">
         <is>
-          <t>Invirtió $164,376 para obtener solo 15 compras (costo $10,958 por venta) con caída de 1,400% en resultados respecto a marzo (de 1 a 15). ROAS de 0 es insostenible con este presupuesto.</t>
+          <t>El anuncio 'Esmaltado Permanente' gastó CLP 164.376 para solo 15 compras, resultando en un CPC de CLP 10.958. Comparado con marzo (1 compra), representa una caída de 1.400% en eficiencia de conversión.</t>
         </is>
       </c>
       <c r="M57" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Pausar anuncio 'Esmaltado Permanente' inmediatamente y reasignar presupuesto a 'Manicurista Integral Carrusel' que opera con costo de $42.</t>
+          <t>→ Acción: Pausar inmediatamente este anuncio y reasignar presupuesto. Analizar si el producto tiene stock o si el landing page tiene errores de conversión.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="50" customHeight="1">
-      <c r="B58" s="78" t="inlineStr">
-        <is>
-          <t>● INSIGHT  Carrusel genera 94% de resultados con 4.5% del presupuesto</t>
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>✦ OPORTUNIDAD  Manicurista Integral Carrusel es estrella oculta</t>
         </is>
       </c>
       <c r="F58" s="75" t="inlineStr">
         <is>
-          <t>El anuncio 'Manicurista Integral Carrusel' con solo $7,688 logró 182 resultados (costo $42), mientras que anuncio de Esmaltado gastó $164,376 en solo 15 ventas. La proporción de eficiencia es 11x mayor.</t>
+          <t>Este anuncio generó 182 link clicks con CPC de CLP 42 y CTR de 3.92%, pero cayó 82.3% en resultados (1.027 en marzo). El hold50 bajo (0.5%) indica problema en retención de video.</t>
         </is>
       </c>
       <c r="M58" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Crear 3 variantes de carrusel similar para otros productos y testear en formato principal de esta campaña.</t>
+          <t>→ Acción: Mantener presupuesto pero cambiar formato de carrusel a video vertical de 9 segundos. Destacar beneficios de certificación en primeros 2 segundos.</t>
         </is>
       </c>
     </row>
@@ -11992,36 +11992,36 @@
       </c>
     </row>
     <row r="61" ht="50" customHeight="1">
-      <c r="B61" s="74" t="inlineStr">
-        <is>
-          <t>✦ OPORTUNIDAD  Segundo video genera 25x ROI respecto a base histórica</t>
+      <c r="B61" s="78" t="inlineStr">
+        <is>
+          <t>● INSIGHT  Formularios generan 76 CLP por lead consistente</t>
         </is>
       </c>
       <c r="F61" s="75" t="inlineStr">
         <is>
-          <t>Anuncio 'Academia Prueba Formularios Segundo video' escaló de 2 leads (marzo) a 514 leads (abril) manteniendo costo controlado de $78 por lead. CTR de 4.15% y hold50 de 9.8% son los mejores de la campaña.</t>
+          <t>Ambos anuncios mantienen CPC estable en CLP 76-78 con alto CTR (4.15-4.33%). Sin embargo, el anuncio 'Cambio 11-07-2025' cayó 9.5% en leads (2.417 vs 2.671 en marzo).</t>
         </is>
       </c>
       <c r="M61" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Aumentar presupuesto de este anuncio de $40,170 a $65,000 (+62%) durante los próximos 7 días para capturar volumen a costo estable.</t>
+          <t>→ Acción: Aumentar presupuesto del anuncio 'Segundo video' de CLP 40.170 a CLP 80.000 (mejor hold50 de 9.8%) y pausar el de Cambio que está perdiendo tracción.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="50" customHeight="1">
-      <c r="B62" s="77" t="inlineStr">
-        <is>
-          <t>⚠ ALERTA  Caída de 9.5% en anuncio principal de formularios</t>
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>✦ OPORTUNIDAD  Academia Segundo Video tiene potencial 5x</t>
         </is>
       </c>
       <c r="F62" s="75" t="inlineStr">
         <is>
-          <t>Anuncio 'Academia Prueba Formularios Cambio 11-07-2025' bajó de 2,671 a 2,417 leads (-254 leads, -9.5%) mientras gasto se mantuvo en $182,818. Esto indica fatiga de audiencia o pérdida de relevancia.</t>
+          <t>Gastó solo CLP 40.170 pero logró 514 leads con CPC de CLP 78 y el mejor hold50 de 9.8%. Es el anuncio con mejor relación eficiencia-presupuesto de toda la cuenta.</t>
         </is>
       </c>
       <c r="M62" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Testear nueva variante de copy/video para este anuncio enfocada en diferenciador versus competencia académica.</t>
+          <t>→ Acción: Duplicar presupuesto de CLP 40.170 a CLP 85.000 esta semana y monitorear CPC para confirmar escalabilidad.</t>
         </is>
       </c>
     </row>
@@ -12035,51 +12035,51 @@
     <row r="65" ht="50" customHeight="1">
       <c r="B65" s="77" t="inlineStr">
         <is>
-          <t>⚠ ALERTA  ROAS promedio crítico de 0.46 en 15 anuncios</t>
+          <t>⚠ ALERTA  BLACK WEEK es único anuncio rentable</t>
         </is>
       </c>
       <c r="F65" s="75" t="inlineStr">
         <is>
-          <t>Campaña invirtió $4,441,047 (86.6% del presupuesto total) para solo 874 compras con ROAS de 0.46 en promedio. Solo 3 anuncios superan ROAS 0.8, indicando 83% de ineficiencia de gasto.</t>
+          <t>De 15 anuncios, solo 'BLACK WEEK INICIO' tiene ROAS superior a 1 (1.18) con 236 compras. Los otros 14 anuncios promedian ROAS 0.27, quemando presupuesto con CPC promedio de CLP 7.894.</t>
         </is>
       </c>
       <c r="M65" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Identificar y pausar anuncios con ROAS &lt;0.2 (Nuevos Esmaltes, Ojos Satinados, Efecto glaseado) liberando $252,550 esta semana.</t>
+          <t>→ Acción: Reasignar CLP 1.500.000 desde anuncios con ROAS &lt; 0.3 hacia BLACK WEEK. Mantener presupuesto solo en: 'Efectos Perlados' (0.46), 'Sedu Tips' (0.42), 'Carrusel Marzo' (0.32).</t>
         </is>
       </c>
     </row>
     <row r="66" ht="50" customHeight="1">
-      <c r="B66" s="78" t="inlineStr">
-        <is>
-          <t>● INSIGHT  BLACK WEEK y Jelly Pop lideran con ROAS 1.18 y 0.93</t>
+      <c r="B66" s="77" t="inlineStr">
+        <is>
+          <t>⚠ ALERTA  Nuevos productos sin conversión (Ojos Satinados, Base Evita)</t>
         </is>
       </c>
       <c r="F66" s="75" t="inlineStr">
         <is>
-          <t>Anuncio 'BLACK WEEK INICIO' generó 236 compras con ROAS 1.18 ($469,274 invertidos), y 'Lanzamiento Jelly Pop' logró ROAS 0.93 (32 compras). Estos dos anuncios representan 30.6% de conversiones con solo 15.5% del presupuesto.</t>
+          <t>'Ojos Satinados Nuevos' gastó CLP 79.423 para solo 4 compras (CPC CLP 19.856) y cayó 89.2% vs marzo. 'Base Evita 2' cayó 69.8% (13 vs 43 compras) con CPC de CLP 10.888.</t>
         </is>
       </c>
       <c r="M66" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Duplicar presupuesto de 'BLACK WEEK INICIO' y 'Jelly Pop' en $150,000 adicionales reasignados de anuncios de bajo ROAS.</t>
+          <t>→ Acción: Pausar ambos anuncios. Verificar si landing page funciona, si el precio es competitivo, o si falta prueba social. Relanzar solo cuando se corrijan estos factores.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="50" customHeight="1">
-      <c r="B67" s="74" t="inlineStr">
-        <is>
-          <t>✦ OPORTUNIDAD  Efectos Perlados con ROAS 0.46 y CTR 2.29% tiene potencial</t>
+      <c r="B67" s="78" t="inlineStr">
+        <is>
+          <t>● INSIGHT  Lanzamiento Jelly Pop emergente con ROAS 0.93</t>
         </is>
       </c>
       <c r="F67" s="75" t="inlineStr">
         <is>
-          <t>Anuncio 'Efectos Perlados en Polvo' mantiene costo controlado de $4,847 por venta y ROAS de 0.46 con CTR superior (2.29%). Hold50 de 6% indica contenido relevante. Con ajuste de targeting podría mejorar significativamente.</t>
+          <t>Nuevo anuncio (sin histórico en marzo) generó 32 compras con ROAS 0.93, el segundo mejor después de BLACK WEEK. CPC de CLP 6.787 es 14% mejor que promedio de campaña.</t>
         </is>
       </c>
       <c r="M67" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Testear segmentación por profesionales de uñas (lookalike custom audience) para este anuncio con presupuesto incremental de $50,000.</t>
+          <t>→ Acción: Aumentar presupuesto de CLP 217.189 a CLP 350.000 y crear 2 variantes adicionales con diferentes ángulos de producto para mantener momentum.</t>
         </is>
       </c>
     </row>
@@ -12093,34 +12093,34 @@
     <row r="70" ht="50" customHeight="1">
       <c r="B70" s="77" t="inlineStr">
         <is>
-          <t>⚠ ALERTA  Caída de 11.8% en anuncio principal con mayor gasto</t>
+          <t>⚠ ALERTA  Se te quebró la uña agosto cayó 11.8% en un mes</t>
         </is>
       </c>
       <c r="F70" s="75" t="inlineStr">
         <is>
-          <t>Anuncio 'Se te quebró la uña agosto' bajó de 25,762 resultados (marzo) a 22,721 (abril) con presupuesto de $99,149. Aunque mantiene excelente CTR de 10.1%, la caída sugiere fatiga creativa con hold50 de 22.1%.</t>
+          <t>El anuncio estrella generó 22.721 clicks pero bajó 1.041 resultados vs marzo (22.721 vs 25.762). A pesar de CPC bajo de CLP 4 y CTR excelente de 10.1%, el hold50 de 22.1% sugiere que el tráfico no convierte en funnel inferior.</t>
         </is>
       </c>
       <c r="M70" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Crear 2 nuevas variantes de copy urgentemente reemplazando 'uña quebrada' por ángulos como 'dureza' o 'brillo' para renovar audiencia.</t>
+          <t>→ Acción: Mantener gasto pero agregar pixel de seguimiento en landing page. Analizar si 22% de usuarios ven el call-to-action o si hay fricción en redirección a Academia/Conversión.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="50" customHeight="1">
-      <c r="B71" s="78" t="inlineStr">
-        <is>
-          <t>● INSIGHT  Campaña de pruebas genera resultados a costo mínimo</t>
+      <c r="B71" s="74" t="inlineStr">
+        <is>
+          <t>✦ OPORTUNIDAD  Anuncios secundarios subinvertidos</t>
         </is>
       </c>
       <c r="F71" s="75" t="inlineStr">
         <is>
-          <t>Con presupuesto de solo $99,381 logró 22,743 resultados (costo $4 por resultado) y CTR promedio de 6.8%. Esta es la campaña más eficiente del portafolio, absorbiendo solo 1.9% del presupuesto.</t>
+          <t>Los 4 anuncios secundarios ('uñas respiran', '5 cosas', 'hannah montana', 'otoño 2026') gastaron solo CLP 232 combinados. Aunque bajo volumen, algunos como 'uñas respiran' tienen CTR de 7.61% y 'otoño 2026' de 4.89%.</t>
         </is>
       </c>
       <c r="M71" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Aumentar presupuesto de esta campaña a $250,000 mensuales para aprovechar eficiencia y generar volumen de tráfico de bajo costo.</t>
+          <t>→ Acción: Asignar CLP 15.000 a cada uno de los 3 mejores anuncios secundarios (excepto hannah montana). Probar si el hook funciona a mayor escala antes de escalar 'Se te quebró'.</t>
         </is>
       </c>
     </row>
@@ -12633,7 +12633,7 @@
     <row r="14" ht="52" customHeight="1">
       <c r="B14" s="73" t="inlineStr">
         <is>
-          <t>Bluesky redujo gasto en 3.6% (de $92,817 a $89,176) pero también disminuyó resultados en 8.1% (de 15,624 a 14,364 clicks). El costo por resultado se mantuvo estable en $6, pero el decrecimiento en conversiones sugiere necesidad de optimización inmediata.</t>
+          <t>Bluesky registró una caída del 8.1% en resultados (15,624 a 14,364 clicks) con gasto reducido 4.0% en abril 2026. El rendimiento por peso invertido se mantuvo estable en $6.21 CPC, pero el mix de anuncios cambió drásticamente con oportunidad de optimización.</t>
         </is>
       </c>
     </row>
@@ -12645,53 +12645,53 @@
       </c>
     </row>
     <row r="17" ht="50" customHeight="1">
-      <c r="B17" s="74" t="inlineStr">
-        <is>
-          <t>✦ OPORTUNIDAD  Diseño Conchitas domina con 77.9% del presupuesto</t>
+      <c r="B17" s="77" t="inlineStr">
+        <is>
+          <t>⚠ ALERTA  Diseño Conchitas concentra 77.9% del presupuesto</t>
         </is>
       </c>
       <c r="F17" s="75" t="inlineStr">
         <is>
-          <t>El anuncio 'Diseño Conchitas' consumió $69,955 (78.4% del gasto) y generó 11,185 clicks (77.9% de resultados), con hold50 de 25% y CTR de 7.1%. Este creative demuestra máxima eficiencia y merece incremento de presupuesto.</t>
+          <t>El anuncio Conchitas consume $69,955 de los $89,176 totales (78.5%) generando 11,185 clicks con CTR de 7.1%. Su hold50 de 25% sugiere retención media pero el costo de $6.25 por click es consistente.</t>
         </is>
       </c>
       <c r="M17" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Aumentar presupuesto diario de 'Diseño Conchitas' en 25-30% esta semana y monitorear ROAS en tiempo real.</t>
+          <t>→ Acción: Auditar la creatividad de Conchitas esta semana para identificar si el alto gasto se debe a bajo rendimiento o alto volumen planificado. Considerar distribuir presupuesto a Floral si CPM es similar.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="50" customHeight="1">
-      <c r="B18" s="77" t="inlineStr">
-        <is>
-          <t>⚠ ALERTA  Caída de 8.1% en resultados totales mes anterior</t>
+      <c r="B18" s="74" t="inlineStr">
+        <is>
+          <t>✦ OPORTUNIDAD  Diseño Floral muestra contracción del 78.6%</t>
         </is>
       </c>
       <c r="F18" s="75" t="inlineStr">
         <is>
-          <t>Los resultados bajaron de 15,624 a 14,364 clicks (-1,260 conversiones, -8.1%) a pesar de mantener costo similar. 'Diseño Floral' cayó 78.6% (de 12,461 a 2,662 resultados) mientras 'Conchitas' creció 253.9%.</t>
+          <t>Floral pasó de 12,461 resultados (marzo) a 2,662 resultados (abril), una caída brutal de 9,799 clicks con presupuesto similar ($15,873). CTR de 7.07% es competitivo pero el hold50 de 13.1% indica fatiga creativa.</t>
         </is>
       </c>
       <c r="M18" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Pausar 'Diseño Floral' por 5 días, revisar copy/imagen y realizar A/B test con variante mejorada antes de relanzar.</t>
+          <t>→ Acción: Reactivar inmediatamente el anuncio Floral con variantes creativas nuevas (ángulos, fondos, paletas) y aumentar presupuesto a $25k para recuperar volumen perdido.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="50" customHeight="1">
       <c r="B19" s="78" t="inlineStr">
         <is>
-          <t>● INSIGHT  Diseño Limón Verano crece 25,350% con bajo gasto</t>
+          <t>● INSIGHT  Limón Verano mostró crecimiento de 25,350%</t>
         </is>
       </c>
       <c r="F19" s="75" t="inlineStr">
         <is>
-          <t>El nuevo anuncio 'diseño limon verano' pasó de 2 a 509 resultados (+255x) invirtiendo solo $3,312 con CTR de 7.58% y hold50 de 18.2%. ROI potencial muy alto con presupuesto mínimo.</t>
+          <t>El anuncio de limón pasó de 2 clicks (marzo) a 509 clicks (abril) con inversión de $3,312 y CTR de 7.58%. Aunque el volumen es bajo, el crecimiento sugiere que el concepto estacional resuena con audiencia.</t>
         </is>
       </c>
       <c r="M19" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Duplicar presupuesto de 'diseño limon verano' a $6,600 esta semana para validar escalabilidad y saturación de audiencia.</t>
+          <t>→ Acción: Aumentar presupuesto de Limón Verano a $15,000 semanales por 2 semanas para validar si es tendencia real o spike puntual. Monitorear daily con umbral de pausa si CPL supera $7.50.</t>
         </is>
       </c>
     </row>
@@ -12725,7 +12725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:R55"/>
+  <dimension ref="B1:R52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -14263,7 +14263,7 @@
     <row r="36" ht="52" customHeight="1">
       <c r="B36" s="73" t="inlineStr">
         <is>
-          <t>Nail Outlet registró un incremento de gasto del 4.2% (1.408M vs 1.352M) pero con caída del 14.4% en resultados (4.302 vs 5.028), evidenciando una eficiencia deteriorada en abril. El ROAS promedio de la marca se redujo significativamente, especialmente en campañas de conversión donde el costo por resultado aumentó en múltiples anuncios.</t>
+          <t>Nail Outlet experimentó una caída del 14.4% en conversiones (de 5.028 a 4.302) pese a aumentar el gasto en 4.2% ($1.408M en abril). La rentabilidad se ha deteriorado significativamente con ROAS promedio bajo en campañas de conversión, requiriendo optimización urgente de creativos y segmentación.</t>
         </is>
       </c>
     </row>
@@ -14277,262 +14277,202 @@
     <row r="39" ht="50" customHeight="1">
       <c r="B39" s="77" t="inlineStr">
         <is>
-          <t>⚠ ALERTA  Caída crítica en Poly Gel Carrusel</t>
+          <t>⚠ ALERTA  Caída crítica en conversiones pack bestseller</t>
         </is>
       </c>
       <c r="F39" s="75" t="inlineStr">
         <is>
-          <t>El anuncio mejor performer cayó 90.4% en conversiones (7 vs 73 resultados) manteniendo inversión de $3.237. Su ROAS de 40.15 indica que sigue siendo rentable pero necesita optimización urgente.</t>
+          <t>Pack Repo 20 Agosto registró una caída del 47.4% en conversiones (de 38 a 20) con inversión similar ($167.478), generando un ROAS de 6.42 pero con eficiencia comprometida. Este fue el mejor anuncio del mes anterior.</t>
         </is>
       </c>
       <c r="M39" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Pausar anuncio, revisar creatividad y audiencia segmentada, reactivar con variación de copy y CTA diferenciado en los próximos 3 días.</t>
+          <t>→ Acción: Analizar cambios en audiencia/creatividad del Pack Repo; considerar renovar videoproducción o segmentar por zona geográfica para recuperar volumen.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="50" customHeight="1">
-      <c r="B40" s="77" t="inlineStr">
-        <is>
-          <t>⚠ ALERTA  Esmaltes French Nail Pro con ROAS negativo</t>
+      <c r="B40" s="74" t="inlineStr">
+        <is>
+          <t>✦ OPORTUNIDAD  Poly Gel Carrusel superhigh performer</t>
         </is>
       </c>
       <c r="F40" s="75" t="inlineStr">
         <is>
-          <t>Gasto de $76.227 generó solo 6 conversiones (vs 14 en marzo) con ROAS de 0.45. Costo por resultado de $12.705 es 3x superior al promedio de campaña.</t>
+          <t>Con solo $3.237 de inversión logró 7 conversiones (ROAS 40.15), pero registra caída de 90.4% vs marzo (73 a 7 resultados). Es el anuncio más eficiente del portafolio.</t>
         </is>
       </c>
       <c r="M40" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Pausar inmediatamente, reasignar presupuesto a Pack Repo 20 Agosto (ROAS 6.42) o Imagen Mesa Nail Pro (ROAS 1.85).</t>
+          <t>→ Acción: Aumentar presupuesto de Poly Gel Carrusel a $15-20K manteniendo segmentación; testear con variaciones de creatividad para replicar performance anterior.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="50" customHeight="1">
-      <c r="B41" s="74" t="inlineStr">
-        <is>
-          <t>✦ OPORTUNIDAD  Pack Repo 20 Agosto sigue siendo rentable</t>
+      <c r="B41" s="78" t="inlineStr">
+        <is>
+          <t>● INSIGHT  Link clicks generan datos sin ROI inmediato</t>
         </is>
       </c>
       <c r="F41" s="75" t="inlineStr">
         <is>
-          <t>A pesar de caída del 47.4% en resultados (20 vs 38), mantiene ROAS de 6.42 con inversión de $167.478. Es el anuncio con mejor relación costo-efectividad en conversión.</t>
+          <t>Ojo de Gato y Como usar Deshidratador generaron 108 clicks con $18.937 pero costo de conversión posterior no se traduce. Hold50 de 6.2% sugiere interés real pero formato incorrecto.</t>
         </is>
       </c>
       <c r="M41" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Aumentar presupuesto diario en 30% y crear 2 variaciones de creatividad para mantener relevancia y recuperar volumen de conversiones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="50" customHeight="1">
-      <c r="B42" s="78" t="inlineStr">
-        <is>
-          <t>● INSIGHT  CTR alto no garantiza conversiones</t>
-        </is>
-      </c>
-      <c r="F42" s="75" t="inlineStr">
-        <is>
-          <t>Imagen primer deshidratador tiene CTR de 2.68% (más alto) pero ROAS de 1.70 con costo de $29.518. Campo de Trabajo tiene CTR de 1.94% con ROAS similar de 1.46.</t>
-        </is>
-      </c>
-      <c r="M42" s="76" t="inlineStr">
-        <is>
-          <t>→ Acción: Implementar pixel de seguimiento mejorado para identificar punto de abandono post-click y optimizar landing page para estos anuncios.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="B44" s="6" t="inlineStr">
+          <t>→ Acción: Separar estos anuncios a campaña de awareness/video view; usar pixel de engagement para remarketing a usuarios con hold50&gt;5%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  💡  TRÁFICO PERFIL INSTAGRAM MKT</t>
         </is>
       </c>
     </row>
+    <row r="44" ht="50" customHeight="1">
+      <c r="B44" s="77" t="inlineStr">
+        <is>
+          <t>⚠ ALERTA  Caída en tráfico pese a bajo costo</t>
+        </is>
+      </c>
+      <c r="F44" s="75" t="inlineStr">
+        <is>
+          <t>Paso a paso Vale Nails cayó 35.4% en clicks (de 2.984 a 1.930) con costo estable ($21). Insta Nail Pro cayó 15.7% (de 1.838 a 2.127 resultados), sugiriendo fatiga de audiencia.</t>
+        </is>
+      </c>
+      <c r="M44" s="76" t="inlineStr">
+        <is>
+          <t>→ Acción: Crear nuevas variantes de creatividad en ambos anuncios; limitar frecuencia a 2 impressiones/usuario/día; testear nuevas audiencias miradores de competencia.</t>
+        </is>
+      </c>
+    </row>
     <row r="45" ht="50" customHeight="1">
-      <c r="B45" s="77" t="inlineStr">
-        <is>
-          <t>⚠ ALERTA  Insta Nail Pro con caída de 15.8%</t>
+      <c r="B45" s="78" t="inlineStr">
+        <is>
+          <t>● INSIGHT  High hold50 indica contenido valuable</t>
         </is>
       </c>
       <c r="F45" s="75" t="inlineStr">
         <is>
-          <t>Generó 2.127 clicks vs 1.838 en marzo (aumento de 15.7%), pero inversión creció de forma no documentada. Hold50 de 19.2% es fuerte pero requiere análisis de conversión posterior.</t>
+          <t>Paso a paso Vale Nails con 4.01% CTR y 10.3% hold50 demuestra que contenido educativo genera engagement, pero no se monetiza adecuadamente.</t>
         </is>
       </c>
       <c r="M45" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Revisar datos de atribución en Google Analytics/Meta Conversions para conectar traffic con compras y calcular ROAS real de esta campaña.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="50" customHeight="1">
-      <c r="B46" s="77" t="inlineStr">
-        <is>
-          <t>⚠ ALERTA  Paso a paso Vale Nails cayó 35.4%</t>
-        </is>
-      </c>
-      <c r="F46" s="75" t="inlineStr">
-        <is>
-          <t>Registró 1.930 clicks vs 2.984 en marzo (caída del 35.4%) con inversión de $41.059. CTR de 4.01% es excelente pero volumen se desmorona.</t>
-        </is>
-      </c>
-      <c r="M46" s="76" t="inlineStr">
-        <is>
-          <t>→ Acción: Reinvertir en este anuncio con nuevo hook visual, cambiar frecuencia de entrega a audiencia similar de mejor calidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="50" customHeight="1">
-      <c r="B47" s="78" t="inlineStr">
-        <is>
-          <t>● INSIGHT  Hold50 alto no se traduce en compras</t>
-        </is>
-      </c>
-      <c r="F47" s="75" t="inlineStr">
-        <is>
-          <t>Ambos anuncios tienen hold50 superior a 10% pero campaña no muestra conversiones. Insta Nail Pro: 19.2% engagement, Paso a paso: 10.3%, indicando buena atracción pero falla en conversión.</t>
-        </is>
-      </c>
-      <c r="M47" s="76" t="inlineStr">
-        <is>
-          <t>→ Acción: Configurar audiences de remarketing basadas en estos clickers y crear anuncios de conversión específicos dentro de 48 horas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="B49" s="6" t="inlineStr">
+          <t>→ Acción: Redirigir esta audiencia con pixel a campaña de conversión del Pack Repo; crear secuencia de remarketing de 7 días antes de saturar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  💡  REMARKETING NAIL OUTLET</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="50" customHeight="1">
-      <c r="B50" s="74" t="inlineStr">
-        <is>
-          <t>✦ OPORTUNIDAD  15% OFF con ROAS de 11.25</t>
-        </is>
-      </c>
-      <c r="F50" s="75" t="inlineStr">
-        <is>
-          <t>Anuncio nuevo que invirtió $20.886 generando 6 conversiones con ROAS de 11.25, el más alto de todas las campañas. Costo unitario de $3.481 es 25% más bajo que promedio.</t>
-        </is>
-      </c>
-      <c r="M50" s="76" t="inlineStr">
-        <is>
-          <t>→ Acción: Aumentar presupuesto diario a $1.000-1.500, crear 2 variaciones (15% OFF vs 20% OFF) y testear durante 7 días.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="50" customHeight="1">
-      <c r="B51" s="78" t="inlineStr">
-        <is>
-          <t>● INSIGHT  Despacho Gratis genera 50% más conversiones</t>
-        </is>
-      </c>
-      <c r="F51" s="75" t="inlineStr">
-        <is>
-          <t>Invirtió $44.220 para 9 conversiones vs 6 del descuento, pero con ROAS inferior (4.85 vs 11.25). Sugiere que mezcla de propuestas de valor es efectiva.</t>
-        </is>
-      </c>
-      <c r="M51" s="76" t="inlineStr">
-        <is>
-          <t>→ Acción: Mantener ambos anuncios activos pero reducir presupuesto de Despacho a $30.000 e incrementar 15% OFF a $35.000 mensuales.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="B53" s="6" t="inlineStr">
+    <row r="48" ht="50" customHeight="1">
+      <c r="B48" s="74" t="inlineStr">
+        <is>
+          <t>✦ OPORTUNIDAD  Remarketing con ROAS doble dígito</t>
+        </is>
+      </c>
+      <c r="F48" s="75" t="inlineStr">
+        <is>
+          <t>15% OFF logró 6 conversiones con ROAS 11.25 ($20.886 gasto), siendo la campaña más rentable del portafolio después del Poly Gel.</t>
+        </is>
+      </c>
+      <c r="M48" s="76" t="inlineStr">
+        <is>
+          <t>→ Acción: Aumentar presupuesto de 15% OFF a $35-40K; crear variante con descuento escalonado (10% vs 15%) para test AB; expandir a carrito abandonado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="50" customHeight="1">
+      <c r="B49" s="78" t="inlineStr">
+        <is>
+          <t>● INSIGHT  Despacho Gratis más volumen menor ROI</t>
+        </is>
+      </c>
+      <c r="F49" s="75" t="inlineStr">
+        <is>
+          <t>Despacho Gratis generó 9 conversiones con ROAS 4.85 ($44.220), doblando volumen pero con menor rentabilidad que 15% OFF, sugiriendo que precio es mayor motivador.</t>
+        </is>
+      </c>
+      <c r="M49" s="76" t="inlineStr">
+        <is>
+          <t>→ Acción: Reducir presupuesto Despacho Gratis a $25K; priorizar 15% OFF como gancho principal; testear combo 10% OFF + envío gratis para segmento ticket bajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  💡  CAMPAÑA CONVERSIÓN CATÁLOGO</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="50" customHeight="1">
-      <c r="B54" s="77" t="inlineStr">
-        <is>
-          <t>⚠ ALERTA  Catálogo nuevo sin historial de performance</t>
-        </is>
-      </c>
-      <c r="F54" s="75" t="inlineStr">
-        <is>
-          <t>Invertido $355.748 (25% del presupuesto total) para apenas 20 conversiones con ROAS de 1.84. Costo por resultado de $17.787 es 4.1x superior al promedio de conversión.</t>
-        </is>
-      </c>
-      <c r="M54" s="76" t="inlineStr">
-        <is>
-          <t>→ Acción: Pausar campaña, solicitar reporte de performance anterior, validar configuración de feed de catálogo y auditar audiencias segmentadas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="50" customHeight="1">
-      <c r="B55" s="77" t="inlineStr">
-        <is>
-          <t>⚠ ALERTA  Hold50 de 0% indica falta de engagement</t>
-        </is>
-      </c>
-      <c r="F55" s="75" t="inlineStr">
-        <is>
-          <t>Pese a CTR aceptable de 1.66%, hold50 es 0%, significando que casi ningún usuario se detiene en el anuncio. Patrón indica creatividad o copy poco atractivos.</t>
-        </is>
-      </c>
-      <c r="M55" s="76" t="inlineStr">
-        <is>
-          <t>→ Acción: Reemplazar creative del catálogo con imágenes de productos high-converting (Pack Repo, Poly Gel) y testar nuevos textos descriptivos.</t>
+    <row r="52" ht="50" customHeight="1">
+      <c r="B52" s="77" t="inlineStr">
+        <is>
+          <t>⚠ ALERTA  Nuevo anuncio catálogo con bajo rendimiento</t>
+        </is>
+      </c>
+      <c r="F52" s="75" t="inlineStr">
+        <is>
+          <t>Único anuncio de catálogo generó solo 20 conversiones con $355.748 de inversión (ROAS 1.84) y 0% hold50, indicando que formato de catálogo dinámico no resonó.</t>
+        </is>
+      </c>
+      <c r="M52" s="76" t="inlineStr">
+        <is>
+          <t>→ Acción: Pausar esta campaña; dividir presupuesto entre Pack Repo (aumentar a $210K) y Black Week (aumentar a $230K) que tienen ROAS 6.42 y 5.57 respectivamente.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="50">
-    <mergeCell ref="F46:L46"/>
+  <mergeCells count="41">
     <mergeCell ref="B40:E40"/>
-    <mergeCell ref="M54:R54"/>
     <mergeCell ref="B26:R26"/>
+    <mergeCell ref="B49:E49"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B35:R35"/>
+    <mergeCell ref="F52:L52"/>
+    <mergeCell ref="B47:R47"/>
     <mergeCell ref="F39:L39"/>
     <mergeCell ref="M40:R40"/>
-    <mergeCell ref="B55:E55"/>
-    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="F48:L48"/>
     <mergeCell ref="B22:R22"/>
+    <mergeCell ref="F49:L49"/>
     <mergeCell ref="B45:E45"/>
-    <mergeCell ref="M46:R46"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B43:R43"/>
     <mergeCell ref="M45:R45"/>
-    <mergeCell ref="M42:R42"/>
-    <mergeCell ref="B54:E54"/>
+    <mergeCell ref="F44:L44"/>
     <mergeCell ref="B2:R2"/>
     <mergeCell ref="M41:R41"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="F54:L54"/>
-    <mergeCell ref="B46:E46"/>
     <mergeCell ref="B1:R1"/>
-    <mergeCell ref="M47:R47"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="F40:L40"/>
-    <mergeCell ref="B44:R44"/>
-    <mergeCell ref="B53:R53"/>
+    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="B48:E48"/>
     <mergeCell ref="B38:R38"/>
-    <mergeCell ref="M50:R50"/>
     <mergeCell ref="B39:E39"/>
-    <mergeCell ref="F55:L55"/>
-    <mergeCell ref="B42:E42"/>
-    <mergeCell ref="F42:L42"/>
-    <mergeCell ref="F51:L51"/>
     <mergeCell ref="F45:L45"/>
-    <mergeCell ref="B49:R49"/>
-    <mergeCell ref="M55:R55"/>
-    <mergeCell ref="F50:L50"/>
+    <mergeCell ref="M44:R44"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B30:R30"/>
     <mergeCell ref="F41:L41"/>
+    <mergeCell ref="M49:R49"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="M52:R52"/>
+    <mergeCell ref="B51:R51"/>
+    <mergeCell ref="M48:R48"/>
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="M39:R39"/>
-    <mergeCell ref="F47:L47"/>
     <mergeCell ref="B5:R5"/>
-    <mergeCell ref="M51:R51"/>
     <mergeCell ref="B36:R36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19190,7 +19130,7 @@
     <row r="90" ht="52" customHeight="1">
       <c r="B90" s="73" t="inlineStr">
         <is>
-          <t>Go Nails experimentó una caída crítica del 88.4% en resultados (de 20,613 a 2,404) en abril 2026 mientras reducía gasto solo 5.7%, indicando un problema sistémico de eficiencia. El ROAS promedio se desplomó y múltiples campañas de conversión generan resultados prácticamente nulos, requiriendo intervención inmediata en estructura de audiencias y creativas.</t>
+          <t>Go Nails experimentó una caída crítica del 88.3% en conversiones (20,613 a 2,404) en abril, aunque redujo gasto un 5.7%. El ROAS se deterioró significativamente en campañas de tráfico, señalando problemas graves en creatividad y targeting.</t>
         </is>
       </c>
     </row>
@@ -19204,34 +19144,34 @@
     <row r="93" ht="50" customHeight="1">
       <c r="B93" s="77" t="inlineStr">
         <is>
-          <t>⚠ ALERTA  Colapso de resultados en anuncios de descuento</t>
+          <t>⚠ ALERTA  Caída de conversiones en remarketing directo</t>
         </is>
       </c>
       <c r="F93" s="75" t="inlineStr">
         <is>
-          <t>El anuncio '15% OFF' cayó de 34 resultados a apenas 1 (97% caída) con CPC de $7,957. El anuncio 'Despacho Gratis' también se desplomó de 108 a 32 resultados (-70.4%), indicando rechazo de audiencia a estas ofertas.</t>
+          <t>El anuncio principal 'Remarketing Go Nails 2024' cayó de 65 a 22 conversiones (66% reducción) con gasto similar (CPC aumentó de 5,863 a 5,863). El anuncio '15% OFF' solo generó 1 conversión versus 34 anteriores.</t>
         </is>
       </c>
       <c r="M93" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Pausar '15% OFF' inmediatamente y testear nuevos hooks de oferta. Segmentar audiencia del anuncio 'Despacho Gratis' por frecuencia de compra previa.</t>
+          <t>→ Acción: Reactivar audiencias de carrito abandonado y revisar pixel de tracking. Testear propuesta de valor diferente al 15% OFF que claramente no convierte.</t>
         </is>
       </c>
     </row>
     <row r="94" ht="50" customHeight="1">
       <c r="B94" s="74" t="inlineStr">
         <is>
-          <t>✦ OPORTUNIDAD  Anuncio principal mantiene eficiencia</t>
+          <t>✦ OPORTUNIDAD  Anuncio 'Despacho Gratis' mantiene eficiencia</t>
         </is>
       </c>
       <c r="F94" s="75" t="inlineStr">
         <is>
-          <t>El anuncio 'Remarketing Go Nails 2024' generó 22 resultados con ROAS 5.24 y CPC $5,863, siendo el mejor performer de la campaña con CTR 1.9%. Representa solo $128,988 del presupuesto de $269,322.</t>
+          <t>Única variante con ROAS saludable de 4.82 y CTR de 1.12%. Aunque cayó de 108 a 32 conversiones, el costo por conversión bajó a $4,137 con mejor CPC.</t>
         </is>
       </c>
       <c r="M94" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Aumentar presupuesto a este anuncio en 50% retirado de los otros dos anuncios de la campaña.</t>
+          <t>→ Acción: Aumentar presupuesto de 'Despacho Gratis' un 40% y replicar estructura creativa a otras campañas de conversión bajo rendimiento.</t>
         </is>
       </c>
     </row>
@@ -19245,51 +19185,51 @@
     <row r="97" ht="50" customHeight="1">
       <c r="B97" s="77" t="inlineStr">
         <is>
-          <t>⚠ ALERTA  Anuncios purchase generan resultados prácticamente nulos</t>
+          <t>⚠ ALERTA  Derrumbe catastrófico en anuncios de compra</t>
         </is>
       </c>
       <c r="F97" s="75" t="inlineStr">
         <is>
-          <t>Los anuncios 'hannah montana 2' ($283,796 gasto, 1 compra, ROAS 0.04) y 'Nueva rutina 4 pasos' ($27,864 gasto, 1 compra) están destruyendo ROI. El primero cayó de 456 a 1 resultado (-99.8%), señalando problema grave de targeting o relevancia.</t>
+          <t>'hannah montana 2' gastó $283,796 por 1 conversión (ROAS 0.04) cayendo de 456 a 1 resultado. 'hannah montana' similar: $55,106 por 1 conversión versus 2,567 anteriores. Pérdida total de $338,902 en estos 2 anuncios.</t>
         </is>
       </c>
       <c r="M97" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Pausar inmediatamente ambos anuncios. Analizar pixel de conversión y verificar que compras se registren correctamente en sistema.</t>
+          <t>→ Acción: Pausar inmediatamente 'hannah montana' y 'hannah montana 2'. Investigar cambios en audiencia/pixel que causaron colapso de 458x en conversiones.</t>
         </is>
       </c>
     </row>
     <row r="98" ht="50" customHeight="1">
-      <c r="B98" s="74" t="inlineStr">
-        <is>
-          <t>✦ OPORTUNIDAD  Link clicks con CTR excepcional sin monetizar</t>
+      <c r="B98" s="78" t="inlineStr">
+        <is>
+          <t>● INSIGHT  Traffic ads generan clics baratos pero sin conversión</t>
         </is>
       </c>
       <c r="F98" s="75" t="inlineStr">
         <is>
-          <t>5 anuncios generan entre 4.3-5.58% CTR con costos de $12-19 por click: 'cotton candy frutilla' (407 clicks), 'tu pareja te debe' (760 clicks), 'popcorn pomo' (25 clicks). Estos demuestran alto interés pero no convierten.</t>
+          <t>'cotton candy frutilla' (CPC $17, CTR 4.3%) generó 407 clics pero 0 conversiones (perdió 208 clicks versus marzo). 'Rutina 4 pasos' mantiene CPC de $15 con buen CTR 4.57% pero sin ROAS medible.</t>
         </is>
       </c>
       <c r="M98" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Crear landing page específica para estos anuncios optimizada para conversión. Testear retargeting dinámico a estos 760+ clickers del anuncio 'tu pareja te debe' con oferta especial.</t>
+          <t>→ Acción: Implementar pixel de compra en landing page. Auditar embudo de conversión post-click (velocidad página, mobile optimization, checkout flow).</t>
         </is>
       </c>
     </row>
     <row r="99" ht="50" customHeight="1">
-      <c r="B99" s="77" t="inlineStr">
-        <is>
-          <t>⚠ ALERTA  Presupuesto mal asignado a anuncios de bajo ROAS</t>
+      <c r="B99" s="74" t="inlineStr">
+        <is>
+          <t>✦ OPORTUNIDAD  Nuevo anuncio 'tu pareja te debe' muestra potencial</t>
         </is>
       </c>
       <c r="F99" s="75" t="inlineStr">
         <is>
-          <t>68% del presupuesto de campaña ($283,796 de $390,118) va a 'hannah montana 2' con ROAS 0.04, mientras anuncios link_click que generan 1,200+ clicks reciben solo 2% del presupuesto.</t>
+          <t>Lanzado en abril sin datos previos: 760 clics por $14,792 (CPC $19), CTR 2.87%. Bajo costo per-click sugiere audiencia receptiva y mensaje relevante.</t>
         </is>
       </c>
       <c r="M99" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Redistribuir presupuesto: reducir anuncios purchase a máximo $20k total, aumentar anuncios link_click a $200k para generar tráfico cualificado.</t>
+          <t>→ Acción: Segmentar 'tu pareja te debe' en audience lookalike. Testear 3 variantes de copy enfocadas en gift/regalo. Aumentar presupuesto a $25k para marzo.</t>
         </is>
       </c>
     </row>
@@ -19303,51 +19243,51 @@
     <row r="102" ht="50" customHeight="1">
       <c r="B102" s="77" t="inlineStr">
         <is>
-          <t>⚠ ALERTA  Caída generalizada de resultados sin reducción proporcional de gasto</t>
+          <t>⚠ ALERTA  Caída del 71% en conversiones de compra</t>
         </is>
       </c>
       <c r="F102" s="75" t="inlineStr">
         <is>
-          <t>Campaña invirtió $5.46M (76.5% del gasto total) y generó solo 715 resultados (-31.3% vs marzo) con CPC promedio $7,642. El anuncio 'Home Spray' solo consumió $1.18M para 91 compras (13% de resultados con 21.7% de gasto).</t>
+          <t>Campaña principal cayó de 2,465 a 715 conversiones pese a invertir $5.46M (76.5% del presupuesto total). 'Home Spray' gastó $1.18M generando solo 91 conversiones (down 27.8%) con ROAS degradado a 2.45.</t>
         </is>
       </c>
       <c r="M102" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Implementar caps de gasto diario máximo $25k por anuncio para evitar desperdicio. Revisar configuración de audiencias: probablemente hay solapamiento y fatiga de audiencia.</t>
+          <t>→ Acción: Pausar 'Home Spray' por 7 días. Renovar creatividades con video formato (actualmente solo imágenes/carruseles). A/B test con propuesta diferente a descuentos.</t>
         </is>
       </c>
     </row>
     <row r="103" ht="50" customHeight="1">
-      <c r="B103" s="74" t="inlineStr">
-        <is>
-          <t>✦ OPORTUNIDAD  Anuncios eficientes con ROAS 4.0+ están subutilizados</t>
+      <c r="B103" s="78" t="inlineStr">
+        <is>
+          <t>● INSIGHT  Anuncios con hold50 alto muestran mayor retención</t>
         </is>
       </c>
       <c r="F103" s="75" t="inlineStr">
         <is>
-          <t>4 anuncios generan ROAS 4.0 o superior con bajo gasto relativo: 'Cremas Sun Kissed' (ROAS 5.0, $68k), 'Imagen Cotton Vlabel' (ROAS 5.0, $293k), 'Imagen Bubble gum' (ROAS 4.1, $100k). Estos representan el 11% del gasto pero eficiencia superior.</t>
+          <t>'4 por 3' (hold50 4.7%, ROAS 3.93), 'Cremas Sun Kissed' (hold50 4.1%, ROAS 5.0) y 'Home Spray' (hold50 6.7%, ROAS 2.45) mantienen mejor performance. Anuncios sin hold50 caen drásticamente.</t>
         </is>
       </c>
       <c r="M103" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Aumentar presupuesto 30-40% a estos 4 anuncios, retirado del anuncio 'Home Spray' (ROAS 2.45) y 'Reel de fragancias' (ROAS 3.03).</t>
+          <t>→ Acción: Priorizar creatividades con 4-7% hold50. Analizar qué elementos en videos retienen 50%+ de audiencia en estos anuncios e implementar en nuevas piezas.</t>
         </is>
       </c>
     </row>
     <row r="104" ht="50" customHeight="1">
-      <c r="B104" s="78" t="inlineStr">
-        <is>
-          <t>● INSIGHT  Nuevos difusores desempeño catastrófico</t>
+      <c r="B104" s="74" t="inlineStr">
+        <is>
+          <t>✦ OPORTUNIDAD  Anuncios de costo bajo con ROAS elite</t>
         </is>
       </c>
       <c r="F104" s="75" t="inlineStr">
         <is>
-          <t>Anuncio 'Nuevos difusores' generó solo 3 resultados con $67,668 gasto (CPC $22,556) y ROAS 1.18, cayendo de 35 a 3 resultados (-91.4%). Peor performer absoluto de la campaña.</t>
+          <t>'Reel cafetería' ($15,267 gasto, ROAS 4.6, CPC $5,089) y 'Imagen Cotton Vlabel' ($293,090, ROAS 5.0, CPC $7,713) muestran eficiencia. Potencial de escala con budget limitado.</t>
         </is>
       </c>
       <c r="M104" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Pausar completamente. Si se relanza, crear creativo completamente nuevo con enfoque en beneficio vs característica del producto.</t>
+          <t>→ Acción: Duplicar presupuesto de 'Reel cafetería' a $30k. Expandir 'Imagen Cotton Vlabel' en 25% (de $293k a $366k) en audiencias lookalike de compradores.</t>
         </is>
       </c>
     </row>
@@ -19361,34 +19301,34 @@
     <row r="107" ht="50" customHeight="1">
       <c r="B107" s="74" t="inlineStr">
         <is>
-          <t>✦ OPORTUNIDAD  ROAS extraordinario en anuncio 'Reel Kit LMM'</t>
+          <t>✦ OPORTUNIDAD  Reel Kit LMM top performer con ROAS 15.27</t>
         </is>
       </c>
       <c r="F107" s="75" t="inlineStr">
         <is>
-          <t>Con apenas $12,363 de gasto, este anuncio generó ROAS 15.27 (5 compras) versus ROAS 3.36 del otro performer. Hold50 de 14.6% indica contenido altamente relevante. Creció de 1 a 5 resultados (+400%).</t>
+          <t>Anuncio menor ($12,363 gasto) generó 5 conversiones con ROAS 15.27 (mayor de toda cuenta). Solo 1 conversión en marzo versus 5 en abril. CPC de $2,473 es 60% más bajo que promedio de conversión.</t>
         </is>
       </c>
       <c r="M107" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Duplicar presupuesto a $25k esta semana. Crear 2-3 variantes de creativo similar basadas en qué elemento del kit genera mayor engagement.</t>
+          <t>→ Acción: Aumentar presupuesto 'Reel Kit LMM' a $50k inmediatamente. Testear 3 variantes del video con hook diferente para mantener hold50 14.6%.</t>
         </is>
       </c>
     </row>
     <row r="108" ht="50" customHeight="1">
       <c r="B108" s="77" t="inlineStr">
         <is>
-          <t>⚠ ALERTA  Anuncio sin tipo de conversión genera costo cero sin datos</t>
+          <t>⚠ ALERTA  Conversión baja en 'Reel esmalte LMM'</t>
         </is>
       </c>
       <c r="F108" s="75" t="inlineStr">
         <is>
-          <t>'Reel de Kit Le Mini' tiene gasto $63 con 0 resultados y 32.1% hold50, pero campo 'tipo' está vacío. Imposible analizar rendimiento o asignar presupuesto.</t>
+          <t>Gastó $60,827 por solo 6 conversiones (CPC $10,138) cayendo de 17 a 6 (64% reducción). Aunque hold50 es alto (19.7%), conversión final es débil.</t>
         </is>
       </c>
       <c r="M108" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Verificar configuración de evento de conversión. Confirmar que anuncio está correctamente etiquetado como 'purchase'. Si sigue sin datos, pausar.</t>
+          <t>→ Acción: Pausar 'Reel esmalte LMM' por 14 días. Crear nueva versión con CTA más agresivo enfocado en urgencia/scarcity. Testear con audiencia más fría.</t>
         </is>
       </c>
     </row>
@@ -19402,51 +19342,51 @@
     <row r="111" ht="50" customHeight="1">
       <c r="B111" s="77" t="inlineStr">
         <is>
-          <t>⚠ ALERTA  Ineficiencia generalizada en generación de tráfico</t>
+          <t>⚠ ALERTA  Costo por click inflado sin conversión final</t>
         </is>
       </c>
       <c r="F111" s="75" t="inlineStr">
         <is>
-          <t>Campaña gastó $935,350 para generar solo 338 link clicks (CPC promedio $2,767), comparado con 'Marketing Go Nails - Trafico Insta' que gastó $390k para 1,285 clicks a $304 CPC. Costo 9x mayor por click.</t>
+          <t>$935,350 generaron 338 clicks (CPC promedio $2,767) pero métrica de compra no está ligada. Anuncios como 'Reel de fragancias' gastaron $523 por solo 2 clicks. Ineficiencia extrema en asignación presupuestaria.</t>
         </is>
       </c>
       <c r="M111" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Auditar audiencias: probablemente está dirigiendo a usuarios fríos. Cambiar targeting a 'Traffico Insta' setup que funciona 9x mejor.</t>
+          <t>→ Acción: Cambiar objetivo de 'link_click' a 'purchase' en todos los anuncios. Auditar UTM tracking para confirmar si conversiones se están registrando correctamente en Meta.</t>
         </is>
       </c>
     </row>
     <row r="112" ht="50" customHeight="1">
-      <c r="B112" s="74" t="inlineStr">
-        <is>
-          <t>✦ OPORTUNIDAD  Dos anuncios purchase con ROAS excepcional</t>
+      <c r="B112" s="78" t="inlineStr">
+        <is>
+          <t>● INSIGHT  Híbridos purchase muestran mejor ROAS</t>
         </is>
       </c>
       <c r="F112" s="75" t="inlineStr">
         <is>
-          <t>Anuncios 'Macbook' (ROAS 9.93, 7 compras, $21.6k) e 'Imagen Bubble gum' (ROAS 5.97, 1 compra, $1.5k) tienen eficiencia purchase-level dentro de campaña link_click.</t>
+          <t>Anuncios con tipo 'purchase' dentro de campaña link_click: 'Macbook' (ROAS 9.93, $21,610 gasto), 'Imagen Bubble gum' (ROAS 5.97) superan 10x el ROAS de puros link_clicks.</t>
         </is>
       </c>
       <c r="M112" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Crear campaña de conversión separada solo con estos 2 creatives. Presupuestar $50k inicialmente en estructura purchase estándar.</t>
+          <t>→ Acción: Convertir todos los anuncios de esta campaña a objetivo 'purchase'. Mantener estructura creativa pero optimizar pixel de compra.</t>
         </is>
       </c>
     </row>
     <row r="113" ht="50" customHeight="1">
-      <c r="B113" s="78" t="inlineStr">
-        <is>
-          <t>● INSIGHT  Anuncios link_click con mejor CPC no generan compras</t>
+      <c r="B113" s="74" t="inlineStr">
+        <is>
+          <t>✦ OPORTUNIDAD  Anuncios de costo ultra-bajo con alto CTR</t>
         </is>
       </c>
       <c r="F113" s="75" t="inlineStr">
         <is>
-          <t>Anuncio 'Hot Chocalate' generó 13 clicks a $35 CPC (excelente), pero $0 en compras. Mismo patrón en 'Fragancias Picnic' (29 clicks, $219 CPC, $0 compras). El tráfico no califica.</t>
+          <t>'Hot Chocalate' ($449 gasto, CTR 4.21%), 'Crema dibujada' ($847), '4 por 3' ($421) generan clicks muy baratos (CPC $35-94). Bajo gasto limita datos pero proporción es prometedora.</t>
         </is>
       </c>
       <c r="M113" s="76" t="inlineStr">
         <is>
-          <t>→ Acción: Implementar pixel de 'ViewContent' más restrictivo. Considerar pausar anuncios link_click y mover presupuesto a campañas purchase con audiencias similares.</t>
+          <t>→ Acción: Incrementar presupuesto en estos 3 anuncios a $5k cada uno. Mantener targeting idéntico pero aumentar reach para validar escalabilidad.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: regenerar Excel con formato compatible con dashboard (marcas mayúsculas, símbolo ▸)
</commit_message>
<xml_diff>
--- a/reportes/Reporte_abril_2026.xlsx
+++ b/reportes/Reporte_abril_2026.xlsx
@@ -927,14 +927,14 @@
     <row r="7" ht="24" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Seducete</t>
+          <t>SEDUCETE</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>▶ Marketing Objetivo Visita Perfil Instagram</t>
+          <t>▸ Marketing Objetivo Visita Perfil Instagram</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1076,7 @@
     <row r="13" ht="22" customHeight="1">
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>▶ Tráfico Web Objetivo Conversión</t>
+          <t>▸ Tráfico Web Objetivo Conversión</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1222,7 @@
     <row r="18" ht="22" customHeight="1">
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>▶ Academia Prueba Formularios</t>
+          <t>▸ Academia Prueba Formularios</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1366,7 @@
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>▶ Conversión Web Ventas</t>
+          <t>▸ Conversión Web Ventas</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
     <row r="47" ht="22" customHeight="1">
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>▶ Campaña Mktg prueba Pau</t>
+          <t>▸ Campaña Mktg prueba Pau</t>
         </is>
       </c>
     </row>
@@ -2958,7 +2958,7 @@
     <row r="55" ht="26" customHeight="1">
       <c r="B55" s="46" t="inlineStr">
         <is>
-          <t>💡  ANÁLISIS CLAUDE — SEDUCETE</t>
+          <t>💡  Análisis Claude — Seducete</t>
         </is>
       </c>
     </row>
@@ -2972,27 +2972,27 @@
     <row r="57" ht="20" customHeight="1">
       <c r="B57" s="48" t="inlineStr">
         <is>
-          <t>CAMPAÑA</t>
+          <t>Campaña</t>
         </is>
       </c>
       <c r="C57" s="48" t="inlineStr">
         <is>
-          <t>TIPO</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="D57" s="48" t="inlineStr">
         <is>
-          <t>TÍTULO DEL HALLAZGO</t>
+          <t>Hallazgo</t>
         </is>
       </c>
       <c r="H57" s="48" t="inlineStr">
         <is>
-          <t>DESCRIPCIÓN</t>
+          <t>Descripción</t>
         </is>
       </c>
       <c r="M57" s="48" t="inlineStr">
         <is>
-          <t>ACCIÓN RECOMENDADA</t>
+          <t>Acción recomendada</t>
         </is>
       </c>
     </row>
@@ -3272,14 +3272,14 @@
     <row r="71" ht="24" customHeight="1">
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Bluesky</t>
+          <t>BLUESKY</t>
         </is>
       </c>
     </row>
     <row r="72" ht="22" customHeight="1">
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>▶ Tráfico Perfil Instagram MKT</t>
+          <t>▸ Tráfico Perfil Instagram MKT</t>
         </is>
       </c>
     </row>
@@ -3529,7 +3529,7 @@
     <row r="79" ht="26" customHeight="1">
       <c r="B79" s="46" t="inlineStr">
         <is>
-          <t>💡  ANÁLISIS CLAUDE — BLUESKY</t>
+          <t>💡  Análisis Claude — Bluesky</t>
         </is>
       </c>
     </row>
@@ -3543,27 +3543,27 @@
     <row r="81" ht="20" customHeight="1">
       <c r="B81" s="48" t="inlineStr">
         <is>
-          <t>CAMPAÑA</t>
+          <t>Campaña</t>
         </is>
       </c>
       <c r="C81" s="48" t="inlineStr">
         <is>
-          <t>TIPO</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="D81" s="48" t="inlineStr">
         <is>
-          <t>TÍTULO DEL HALLAZGO</t>
+          <t>Hallazgo</t>
         </is>
       </c>
       <c r="H81" s="48" t="inlineStr">
         <is>
-          <t>DESCRIPCIÓN</t>
+          <t>Descripción</t>
         </is>
       </c>
       <c r="M81" s="48" t="inlineStr">
         <is>
-          <t>ACCIÓN RECOMENDADA</t>
+          <t>Acción recomendada</t>
         </is>
       </c>
     </row>
@@ -3643,14 +3643,14 @@
     <row r="87" ht="24" customHeight="1">
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Nail Outlet</t>
+          <t>NAIL OUTLET</t>
         </is>
       </c>
     </row>
     <row r="88" ht="22" customHeight="1">
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>▶ Objetivo Conversión Ventas</t>
+          <t>▸ Objetivo Conversión Ventas</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
     <row r="106" ht="22" customHeight="1">
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>▶ Tráfico Perfil Instagram MKT</t>
+          <t>▸ Tráfico Perfil Instagram MKT</t>
         </is>
       </c>
     </row>
@@ -4706,7 +4706,7 @@
     <row r="111" ht="22" customHeight="1">
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>▶ Remarketing Nail Outlet</t>
+          <t>▸ Remarketing Nail Outlet</t>
         </is>
       </c>
     </row>
@@ -4850,7 +4850,7 @@
     <row r="116" ht="22" customHeight="1">
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>▶ Campaña Conversión Catálogo</t>
+          <t>▸ Campaña Conversión Catálogo</t>
         </is>
       </c>
     </row>
@@ -4926,7 +4926,7 @@
     <row r="120" ht="26" customHeight="1">
       <c r="B120" s="46" t="inlineStr">
         <is>
-          <t>💡  ANÁLISIS CLAUDE — NAIL OUTLET</t>
+          <t>💡  Análisis Claude — Nail Outlet</t>
         </is>
       </c>
     </row>
@@ -4940,27 +4940,27 @@
     <row r="122" ht="20" customHeight="1">
       <c r="B122" s="48" t="inlineStr">
         <is>
-          <t>CAMPAÑA</t>
+          <t>Campaña</t>
         </is>
       </c>
       <c r="C122" s="48" t="inlineStr">
         <is>
-          <t>TIPO</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="D122" s="48" t="inlineStr">
         <is>
-          <t>TÍTULO DEL HALLAZGO</t>
+          <t>Hallazgo</t>
         </is>
       </c>
       <c r="H122" s="48" t="inlineStr">
         <is>
-          <t>DESCRIPCIÓN</t>
+          <t>Descripción</t>
         </is>
       </c>
       <c r="M122" s="48" t="inlineStr">
         <is>
-          <t>ACCIÓN RECOMENDADA</t>
+          <t>Acción recomendada</t>
         </is>
       </c>
     </row>
@@ -5190,14 +5190,14 @@
     <row r="134" ht="24" customHeight="1">
       <c r="B134" s="4" t="inlineStr">
         <is>
-          <t>Go Nails</t>
+          <t>GO NAILS</t>
         </is>
       </c>
     </row>
     <row r="135" ht="22" customHeight="1">
       <c r="B135" s="5" t="inlineStr">
         <is>
-          <t>▶ Remarketing Go Nails 2024</t>
+          <t>▸ Remarketing Go Nails 2024</t>
         </is>
       </c>
     </row>
@@ -5405,7 +5405,7 @@
     <row r="141" ht="22" customHeight="1">
       <c r="B141" s="5" t="inlineStr">
         <is>
-          <t>▶ Marketing Go Nails - Trafico Insta</t>
+          <t>▸ Marketing Go Nails - Trafico Insta</t>
         </is>
       </c>
     </row>
@@ -5937,7 +5937,7 @@
     <row r="153" ht="22" customHeight="1">
       <c r="B153" s="5" t="inlineStr">
         <is>
-          <t>▶ Campaña principal de Conversión</t>
+          <t>▸ Campaña principal de Conversión</t>
         </is>
       </c>
     </row>
@@ -7811,7 +7811,7 @@
     <row r="187" ht="22" customHeight="1">
       <c r="B187" s="5" t="inlineStr">
         <is>
-          <t>▶ Campaña Secundaria LMM</t>
+          <t>▸ Campaña Secundaria LMM</t>
         </is>
       </c>
     </row>
@@ -8009,7 +8009,7 @@
     <row r="193" ht="22" customHeight="1">
       <c r="B193" s="5" t="inlineStr">
         <is>
-          <t>▶ Campaña Conversión Catálogo</t>
+          <t>▸ Campaña Conversión Catálogo</t>
         </is>
       </c>
     </row>
@@ -9543,7 +9543,7 @@
     <row r="222" ht="26" customHeight="1">
       <c r="B222" s="46" t="inlineStr">
         <is>
-          <t>💡  ANÁLISIS CLAUDE — GO NAILS</t>
+          <t>💡  Análisis Claude — Go Nails</t>
         </is>
       </c>
     </row>
@@ -9557,27 +9557,27 @@
     <row r="224" ht="20" customHeight="1">
       <c r="B224" s="48" t="inlineStr">
         <is>
-          <t>CAMPAÑA</t>
+          <t>Campaña</t>
         </is>
       </c>
       <c r="C224" s="48" t="inlineStr">
         <is>
-          <t>TIPO</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="D224" s="48" t="inlineStr">
         <is>
-          <t>TÍTULO DEL HALLAZGO</t>
+          <t>Hallazgo</t>
         </is>
       </c>
       <c r="H224" s="48" t="inlineStr">
         <is>
-          <t>DESCRIPCIÓN</t>
+          <t>Descripción</t>
         </is>
       </c>
       <c r="M224" s="48" t="inlineStr">
         <is>
-          <t>ACCIÓN RECOMENDADA</t>
+          <t>Acción recomendada</t>
         </is>
       </c>
     </row>

</xml_diff>